<commit_message>
Fix weekend coloring: remove hard-coded gray, rely on conditional formatting
3月の土日に直接塗られていた固定の灰色を消去し、土日の着色を
条件付き書式（自動）に一本化。月を変えても土日以外が塗られない。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cr2RrSG9u7J1m38g1q19AJ
</commit_message>
<xml_diff>
--- a/cea765fb-________.xlsx
+++ b/cea765fb-________.xlsx
@@ -252,12 +252,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -740,26 +738,26 @@
         <f>DATE(VALUE(LEFT($A$2,FIND("年度",$A$2)-1)),VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),1)</f>
         <v/>
       </c>
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="21" t="n"/>
-      <c r="E4" s="21" t="n"/>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="24" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5" ht="21" customHeight="1" s="19">
-      <c r="A5" s="24">
+      <c r="A5" s="23">
         <f>IF($A4="","",IF(MONTH($A4+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A4+1,""))</f>
         <v/>
       </c>
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="21" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -768,14 +766,14 @@
       <c r="G5" s="4" t="n"/>
     </row>
     <row r="6" ht="21" customHeight="1" s="19">
-      <c r="A6" s="24">
+      <c r="A6" s="23">
         <f>IF($A5="","",IF(MONTH($A5+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A5+1,""))</f>
         <v/>
       </c>
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="8" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="21" t="n"/>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -784,14 +782,14 @@
       <c r="G6" s="4" t="n"/>
     </row>
     <row r="7" ht="21" customHeight="1" s="19">
-      <c r="A7" s="24">
+      <c r="A7" s="23">
         <f>IF($A6="","",IF(MONTH($A6+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A6+1,""))</f>
         <v/>
       </c>
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="8" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="21" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="24" t="n"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -800,14 +798,14 @@
       <c r="G7" s="4" t="n"/>
     </row>
     <row r="8" ht="21" customHeight="1" s="19">
-      <c r="A8" s="24">
+      <c r="A8" s="23">
         <f>IF($A7="","",IF(MONTH($A7+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A7+1,""))</f>
         <v/>
       </c>
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="8" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="24" t="n"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -816,14 +814,14 @@
       <c r="G8" s="4" t="n"/>
     </row>
     <row r="9" ht="21" customHeight="1" s="19">
-      <c r="A9" s="24">
+      <c r="A9" s="23">
         <f>IF($A8="","",IF(MONTH($A8+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A8+1,""))</f>
         <v/>
       </c>
       <c r="B9" s="9" t="n"/>
       <c r="C9" s="8" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -836,42 +834,42 @@
         <f>IF($A9="","",IF(MONTH($A9+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A9+1,""))</f>
         <v/>
       </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
     </row>
     <row r="11" ht="21" customHeight="1" s="19">
       <c r="A11" s="23">
         <f>IF($A10="","",IF(MONTH($A10+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A10+1,""))</f>
         <v/>
       </c>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1" s="19">
-      <c r="A12" s="24">
+      <c r="A12" s="23">
         <f>IF($A11="","",IF(MONTH($A11+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A11+1,""))</f>
         <v/>
       </c>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="8" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
       <c r="F12" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -880,14 +878,14 @@
       <c r="G12" s="4" t="n"/>
     </row>
     <row r="13" ht="21" customHeight="1" s="19">
-      <c r="A13" s="24">
+      <c r="A13" s="23">
         <f>IF($A12="","",IF(MONTH($A12+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A12+1,""))</f>
         <v/>
       </c>
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="8" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
       <c r="F13" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -896,14 +894,14 @@
       <c r="G13" s="4" t="n"/>
     </row>
     <row r="14" ht="21" customHeight="1" s="19">
-      <c r="A14" s="24">
+      <c r="A14" s="23">
         <f>IF($A13="","",IF(MONTH($A13+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A13+1,""))</f>
         <v/>
       </c>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="8" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
       <c r="F14" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -912,14 +910,14 @@
       <c r="G14" s="4" t="n"/>
     </row>
     <row r="15" ht="21" customHeight="1" s="19">
-      <c r="A15" s="24">
+      <c r="A15" s="23">
         <f>IF($A14="","",IF(MONTH($A14+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A14+1,""))</f>
         <v/>
       </c>
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="8" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="21" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
       <c r="F15" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -928,14 +926,14 @@
       <c r="G15" s="4" t="n"/>
     </row>
     <row r="16" ht="21" customHeight="1" s="19">
-      <c r="A16" s="24">
+      <c r="A16" s="23">
         <f>IF($A15="","",IF(MONTH($A15+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A15+1,""))</f>
         <v/>
       </c>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="8" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="21" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
       <c r="F16" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -948,42 +946,42 @@
         <f>IF($A16="","",IF(MONTH($A16+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A16+1,""))</f>
         <v/>
       </c>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18" ht="21" customHeight="1" s="19">
       <c r="A18" s="23">
         <f>IF($A17="","",IF(MONTH($A17+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A17+1,""))</f>
         <v/>
       </c>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G18" s="16" t="n"/>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
     </row>
     <row r="19" ht="21" customHeight="1" s="19">
-      <c r="A19" s="24">
+      <c r="A19" s="23">
         <f>IF($A18="","",IF(MONTH($A18+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A18+1,""))</f>
         <v/>
       </c>
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="8" t="n"/>
-      <c r="D19" s="21" t="n"/>
-      <c r="E19" s="21" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
       <c r="F19" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -992,14 +990,14 @@
       <c r="G19" s="4" t="n"/>
     </row>
     <row r="20" ht="21" customHeight="1" s="19">
-      <c r="A20" s="24">
+      <c r="A20" s="23">
         <f>IF($A19="","",IF(MONTH($A19+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A19+1,""))</f>
         <v/>
       </c>
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="8" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="E20" s="21" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
       <c r="F20" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1008,14 +1006,14 @@
       <c r="G20" s="4" t="n"/>
     </row>
     <row r="21" ht="21" customHeight="1" s="19">
-      <c r="A21" s="24">
+      <c r="A21" s="23">
         <f>IF($A20="","",IF(MONTH($A20+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A20+1,""))</f>
         <v/>
       </c>
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="8" t="n"/>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="21" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1024,14 +1022,14 @@
       <c r="G21" s="4" t="n"/>
     </row>
     <row r="22" ht="21" customHeight="1" s="19">
-      <c r="A22" s="24">
+      <c r="A22" s="23">
         <f>IF($A21="","",IF(MONTH($A21+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A21+1,""))</f>
         <v/>
       </c>
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1040,14 +1038,14 @@
       <c r="G22" s="4" t="n"/>
     </row>
     <row r="23" ht="21" customHeight="1" s="19">
-      <c r="A23" s="24">
+      <c r="A23" s="23">
         <f>IF($A22="","",IF(MONTH($A22+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A22+1,""))</f>
         <v/>
       </c>
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="21" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
       <c r="F23" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1060,42 +1058,42 @@
         <f>IF($A23="","",IF(MONTH($A23+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A23+1,""))</f>
         <v/>
       </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="21" t="n"/>
-      <c r="E24" s="21" t="n"/>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="n"/>
+      <c r="B24" s="9" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
     </row>
     <row r="25" ht="21" customHeight="1" s="19">
       <c r="A25" s="23">
         <f>IF($A24="","",IF(MONTH($A24+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A24+1,""))</f>
         <v/>
       </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="21" t="n"/>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="n"/>
+      <c r="B25" s="9" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26" ht="21" customHeight="1" s="19">
-      <c r="A26" s="24">
+      <c r="A26" s="23">
         <f>IF($A25="","",IF(MONTH($A25+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A25+1,""))</f>
         <v/>
       </c>
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="21" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
       <c r="F26" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1104,14 +1102,14 @@
       <c r="G26" s="4" t="n"/>
     </row>
     <row r="27" ht="21" customHeight="1" s="19">
-      <c r="A27" s="24">
+      <c r="A27" s="23">
         <f>IF($A26="","",IF(MONTH($A26+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A26+1,""))</f>
         <v/>
       </c>
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="21" t="n"/>
-      <c r="E27" s="21" t="n"/>
+      <c r="D27" s="24" t="n"/>
+      <c r="E27" s="24" t="n"/>
       <c r="F27" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1120,14 +1118,14 @@
       <c r="G27" s="4" t="n"/>
     </row>
     <row r="28" ht="21" customHeight="1" s="19">
-      <c r="A28" s="24">
+      <c r="A28" s="23">
         <f>IF($A27="","",IF(MONTH($A27+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A27+1,""))</f>
         <v/>
       </c>
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="21" t="n"/>
-      <c r="E28" s="21" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
       <c r="F28" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1136,14 +1134,14 @@
       <c r="G28" s="4" t="n"/>
     </row>
     <row r="29" ht="21" customHeight="1" s="19">
-      <c r="A29" s="24">
+      <c r="A29" s="23">
         <f>IF($A28="","",IF(MONTH($A28+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A28+1,""))</f>
         <v/>
       </c>
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="8" t="n"/>
-      <c r="D29" s="21" t="n"/>
-      <c r="E29" s="21" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
       <c r="F29" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1152,14 +1150,14 @@
       <c r="G29" s="4" t="n"/>
     </row>
     <row r="30" ht="21" customHeight="1" s="19">
-      <c r="A30" s="24">
+      <c r="A30" s="23">
         <f>IF($A29="","",IF(MONTH($A29+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A29+1,""))</f>
         <v/>
       </c>
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="21" t="n"/>
-      <c r="E30" s="21" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1172,42 +1170,42 @@
         <f>IF($A30="","",IF(MONTH($A30+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A30+1,""))</f>
         <v/>
       </c>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="21" t="n"/>
-      <c r="E31" s="21" t="n"/>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G31" s="16" t="n"/>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32" ht="21" customHeight="1" s="19">
       <c r="A32" s="23">
         <f>IF($A31="","",IF(MONTH($A31+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A31+1,""))</f>
         <v/>
       </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="21" t="n"/>
-      <c r="E32" s="21" t="n"/>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G32" s="16" t="n"/>
+      <c r="B32" s="9" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n"/>
     </row>
     <row r="33" ht="21" customHeight="1" s="19">
-      <c r="A33" s="24">
+      <c r="A33" s="23">
         <f>IF($A32="","",IF(MONTH($A32+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A32+1,""))</f>
         <v/>
       </c>
       <c r="B33" s="9" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="21" t="n"/>
-      <c r="E33" s="21" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
       <c r="F33" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1216,14 +1214,14 @@
       <c r="G33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="24">
+      <c r="A34" s="23">
         <f>IF($A33="","",IF(MONTH($A33+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A33+1,""))</f>
         <v/>
       </c>
       <c r="B34" s="9" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="21" t="n"/>
-      <c r="E34" s="21" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1360,26 +1358,26 @@
         <f>DATE(VALUE(LEFT($A$2,FIND("年度",$A$2)-1)),VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),1)</f>
         <v/>
       </c>
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="21" t="n"/>
-      <c r="E4" s="21" t="n"/>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="24" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5" ht="21" customHeight="1" s="19">
-      <c r="A5" s="24">
+      <c r="A5" s="23">
         <f>IF($A4="","",IF(MONTH($A4+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A4+1,""))</f>
         <v/>
       </c>
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="21" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1388,14 +1386,14 @@
       <c r="G5" s="4" t="n"/>
     </row>
     <row r="6" ht="21" customHeight="1" s="19">
-      <c r="A6" s="24">
+      <c r="A6" s="23">
         <f>IF($A5="","",IF(MONTH($A5+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A5+1,""))</f>
         <v/>
       </c>
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="8" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="21" t="n"/>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1404,14 +1402,14 @@
       <c r="G6" s="4" t="n"/>
     </row>
     <row r="7" ht="21" customHeight="1" s="19">
-      <c r="A7" s="24">
+      <c r="A7" s="23">
         <f>IF($A6="","",IF(MONTH($A6+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A6+1,""))</f>
         <v/>
       </c>
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="8" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="21" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="24" t="n"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1420,14 +1418,14 @@
       <c r="G7" s="4" t="n"/>
     </row>
     <row r="8" ht="21" customHeight="1" s="19">
-      <c r="A8" s="24">
+      <c r="A8" s="23">
         <f>IF($A7="","",IF(MONTH($A7+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A7+1,""))</f>
         <v/>
       </c>
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="8" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="24" t="n"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1436,14 +1434,14 @@
       <c r="G8" s="4" t="n"/>
     </row>
     <row r="9" ht="21" customHeight="1" s="19">
-      <c r="A9" s="24">
+      <c r="A9" s="23">
         <f>IF($A8="","",IF(MONTH($A8+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A8+1,""))</f>
         <v/>
       </c>
       <c r="B9" s="9" t="n"/>
       <c r="C9" s="8" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1456,42 +1454,42 @@
         <f>IF($A9="","",IF(MONTH($A9+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A9+1,""))</f>
         <v/>
       </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
     </row>
     <row r="11" ht="21" customHeight="1" s="19">
       <c r="A11" s="23">
         <f>IF($A10="","",IF(MONTH($A10+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A10+1,""))</f>
         <v/>
       </c>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1" s="19">
-      <c r="A12" s="24">
+      <c r="A12" s="23">
         <f>IF($A11="","",IF(MONTH($A11+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A11+1,""))</f>
         <v/>
       </c>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="8" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
       <c r="F12" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1500,14 +1498,14 @@
       <c r="G12" s="4" t="n"/>
     </row>
     <row r="13" ht="21" customHeight="1" s="19">
-      <c r="A13" s="24">
+      <c r="A13" s="23">
         <f>IF($A12="","",IF(MONTH($A12+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A12+1,""))</f>
         <v/>
       </c>
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="8" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
       <c r="F13" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1516,14 +1514,14 @@
       <c r="G13" s="4" t="n"/>
     </row>
     <row r="14" ht="21" customHeight="1" s="19">
-      <c r="A14" s="24">
+      <c r="A14" s="23">
         <f>IF($A13="","",IF(MONTH($A13+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A13+1,""))</f>
         <v/>
       </c>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="8" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
       <c r="F14" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1532,14 +1530,14 @@
       <c r="G14" s="4" t="n"/>
     </row>
     <row r="15" ht="21" customHeight="1" s="19">
-      <c r="A15" s="24">
+      <c r="A15" s="23">
         <f>IF($A14="","",IF(MONTH($A14+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A14+1,""))</f>
         <v/>
       </c>
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="8" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="21" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
       <c r="F15" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1548,14 +1546,14 @@
       <c r="G15" s="4" t="n"/>
     </row>
     <row r="16" ht="21" customHeight="1" s="19">
-      <c r="A16" s="24">
+      <c r="A16" s="23">
         <f>IF($A15="","",IF(MONTH($A15+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A15+1,""))</f>
         <v/>
       </c>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="8" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="21" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
       <c r="F16" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1568,42 +1566,42 @@
         <f>IF($A16="","",IF(MONTH($A16+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A16+1,""))</f>
         <v/>
       </c>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18" ht="21" customHeight="1" s="19">
       <c r="A18" s="23">
         <f>IF($A17="","",IF(MONTH($A17+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A17+1,""))</f>
         <v/>
       </c>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G18" s="16" t="n"/>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
     </row>
     <row r="19" ht="21" customHeight="1" s="19">
-      <c r="A19" s="24">
+      <c r="A19" s="23">
         <f>IF($A18="","",IF(MONTH($A18+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A18+1,""))</f>
         <v/>
       </c>
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="8" t="n"/>
-      <c r="D19" s="21" t="n"/>
-      <c r="E19" s="21" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
       <c r="F19" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1612,14 +1610,14 @@
       <c r="G19" s="4" t="n"/>
     </row>
     <row r="20" ht="21" customHeight="1" s="19">
-      <c r="A20" s="24">
+      <c r="A20" s="23">
         <f>IF($A19="","",IF(MONTH($A19+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A19+1,""))</f>
         <v/>
       </c>
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="8" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="E20" s="21" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
       <c r="F20" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1628,14 +1626,14 @@
       <c r="G20" s="4" t="n"/>
     </row>
     <row r="21" ht="21" customHeight="1" s="19">
-      <c r="A21" s="24">
+      <c r="A21" s="23">
         <f>IF($A20="","",IF(MONTH($A20+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A20+1,""))</f>
         <v/>
       </c>
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="8" t="n"/>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="21" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1644,14 +1642,14 @@
       <c r="G21" s="4" t="n"/>
     </row>
     <row r="22" ht="21" customHeight="1" s="19">
-      <c r="A22" s="24">
+      <c r="A22" s="23">
         <f>IF($A21="","",IF(MONTH($A21+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A21+1,""))</f>
         <v/>
       </c>
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="8" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1660,14 +1658,14 @@
       <c r="G22" s="4" t="n"/>
     </row>
     <row r="23" ht="21" customHeight="1" s="19">
-      <c r="A23" s="24">
+      <c r="A23" s="23">
         <f>IF($A22="","",IF(MONTH($A22+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A22+1,""))</f>
         <v/>
       </c>
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="8" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="21" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
       <c r="F23" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1680,42 +1678,42 @@
         <f>IF($A23="","",IF(MONTH($A23+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A23+1,""))</f>
         <v/>
       </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="21" t="n"/>
-      <c r="E24" s="21" t="n"/>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="n"/>
+      <c r="B24" s="9" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
     </row>
     <row r="25" ht="21" customHeight="1" s="19">
       <c r="A25" s="23">
         <f>IF($A24="","",IF(MONTH($A24+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A24+1,""))</f>
         <v/>
       </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="21" t="n"/>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="n"/>
+      <c r="B25" s="9" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26" ht="21" customHeight="1" s="19">
-      <c r="A26" s="24">
+      <c r="A26" s="23">
         <f>IF($A25="","",IF(MONTH($A25+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A25+1,""))</f>
         <v/>
       </c>
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="21" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
       <c r="F26" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1724,14 +1722,14 @@
       <c r="G26" s="4" t="n"/>
     </row>
     <row r="27" ht="21" customHeight="1" s="19">
-      <c r="A27" s="24">
+      <c r="A27" s="23">
         <f>IF($A26="","",IF(MONTH($A26+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A26+1,""))</f>
         <v/>
       </c>
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="8" t="n"/>
-      <c r="D27" s="21" t="n"/>
-      <c r="E27" s="21" t="n"/>
+      <c r="D27" s="24" t="n"/>
+      <c r="E27" s="24" t="n"/>
       <c r="F27" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1740,14 +1738,14 @@
       <c r="G27" s="4" t="n"/>
     </row>
     <row r="28" ht="21" customHeight="1" s="19">
-      <c r="A28" s="24">
+      <c r="A28" s="23">
         <f>IF($A27="","",IF(MONTH($A27+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A27+1,""))</f>
         <v/>
       </c>
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="8" t="n"/>
-      <c r="D28" s="21" t="n"/>
-      <c r="E28" s="21" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
       <c r="F28" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1756,14 +1754,14 @@
       <c r="G28" s="4" t="n"/>
     </row>
     <row r="29" ht="21" customHeight="1" s="19">
-      <c r="A29" s="24">
+      <c r="A29" s="23">
         <f>IF($A28="","",IF(MONTH($A28+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A28+1,""))</f>
         <v/>
       </c>
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="8" t="n"/>
-      <c r="D29" s="21" t="n"/>
-      <c r="E29" s="21" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
       <c r="F29" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1772,14 +1770,14 @@
       <c r="G29" s="4" t="n"/>
     </row>
     <row r="30" ht="21" customHeight="1" s="19">
-      <c r="A30" s="24">
+      <c r="A30" s="23">
         <f>IF($A29="","",IF(MONTH($A29+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A29+1,""))</f>
         <v/>
       </c>
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="21" t="n"/>
-      <c r="E30" s="21" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1792,42 +1790,42 @@
         <f>IF($A30="","",IF(MONTH($A30+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A30+1,""))</f>
         <v/>
       </c>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="21" t="n"/>
-      <c r="E31" s="21" t="n"/>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G31" s="16" t="n"/>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32" ht="21" customHeight="1" s="19">
       <c r="A32" s="23">
         <f>IF($A31="","",IF(MONTH($A31+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A31+1,""))</f>
         <v/>
       </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="21" t="n"/>
-      <c r="E32" s="21" t="n"/>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G32" s="16" t="n"/>
+      <c r="B32" s="9" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n"/>
     </row>
     <row r="33" ht="21" customHeight="1" s="19">
-      <c r="A33" s="24">
+      <c r="A33" s="23">
         <f>IF($A32="","",IF(MONTH($A32+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A32+1,""))</f>
         <v/>
       </c>
       <c r="B33" s="9" t="n"/>
       <c r="C33" s="8" t="n"/>
-      <c r="D33" s="21" t="n"/>
-      <c r="E33" s="21" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
       <c r="F33" s="4" t="inlineStr">
         <is>
           <t>/</t>
@@ -1836,14 +1834,14 @@
       <c r="G33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="24">
+      <c r="A34" s="23">
         <f>IF($A33="","",IF(MONTH($A33+1)=VALUE(SUBSTITUTE(SUBSTITUTE(LEFT($A$1,FIND("月度",$A$1)-1),"　","")," ","")),$A33+1,""))</f>
         <v/>
       </c>
       <c r="B34" s="9" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="21" t="n"/>
-      <c r="E34" s="21" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
           <t>/</t>

</xml_diff>